<commit_message>
chore: 全项目由临时名 smart-agent 更名为 QIO
- 产品名/标识: Smart Agent -> QIO, com.smartagent.app -> com.qio.app, APP_NAME/SERVICE_NAME/FastAPI title -> qio

- 环境变量前缀: SMART_AGENT_* -> QIO_* (PORT/DATA_DIR/HOST/LOG/DB/ARCHIVE/KEY_*)

- sidecar: smart-agent-backend -> qio-backend (spec / externalBin / 构建脚本 / 磁盘产物)

- 数据目录: %APPDATA%/smart-agent -> %APPDATA%/qio; npm/cargo 包名同步

- 文档与 e2e 清单 xlsx 同步; .gitignore 增加 scripts/.e2e-pids
</commit_message>
<xml_diff>
--- a/docs/e2e-test-checklist.xlsx
+++ b/docs/e2e-test-checklist.xlsx
@@ -466,14 +466,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Smart Agent 端到端测试清单</t>
+          <t>QIO 端到端测试清单</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>项目：Smart Agent · 版本 v0.7 · 用例总数 30 · 生成日期 2026-08-03</t>
+          <t>项目：QIO · 版本 v0.7 · 用例总数 30 · 生成日期 2026-08-03</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>Smart Agent 端到端测试清单 · 使用说明</t>
+          <t>QIO 端到端测试清单 · 使用说明</t>
         </is>
       </c>
       <c r="B1" s="19" t="str"/>

</xml_diff>